<commit_message>
Add TC_LOGIN_001 login page display check
</commit_message>
<xml_diff>
--- a/test_cases/login_test_cases.xlsx
+++ b/test_cases/login_test_cases.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,48 @@
       <c r="J1" t="inlineStr">
         <is>
           <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Ki?m tra trang ??ng nh?p hi?n th? ??y ??</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>M? ???c website</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>M? URL ??ng nh?p; quan s?t ti?u ??, t?n ??ng nh?p, m?t kh?u v? n?t ??ng nh?p</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Hi?n th? ??ng trang ??ng nh?p c?ng c?c tr??ng v? n?t c?n thi?t</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>page_load</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Not Run</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add TC_LOGIN_002 empty credentials case
</commit_message>
<xml_diff>
--- a/test_cases/login_test_cases.xlsx
+++ b/test_cases/login_test_cases.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -508,7 +508,49 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>??ng nh?p khi b? tr?ng c? t?n ??ng nh?p v? m?t kh?u</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>?ang ? trang ??ng nh?p</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>?? tr?ng hai tr??ng; nh?n ??ng nh?p</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Kh?ng v?o ???c ?ng d?ng; ti?p t?c ? trang ??ng nh?p</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>submit_empty</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add TC_LOGIN_003 username only case
</commit_message>
<xml_diff>
--- a/test_cases/login_test_cases.xlsx
+++ b/test_cases/login_test_cases.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -549,6 +549,53 @@
         </is>
       </c>
       <c r="J3" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>??ng nh?p ch? nh?p t?n ??ng nh?p</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>?ang ? trang ??ng nh?p</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>kiemthu_automation</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Nh?p t?n ??ng nh?p; ?? tr?ng m?t kh?u; nh?n ??ng nh?p</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Kh?ng v?o ???c ?ng d?ng; ti?p t?c ? trang ??ng nh?p</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>submit_username_only</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>

</xml_diff>

<commit_message>
Add TC_LOGIN_004 password only case
</commit_message>
<xml_diff>
--- a/test_cases/login_test_cases.xlsx
+++ b/test_cases/login_test_cases.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -596,6 +596,53 @@
         </is>
       </c>
       <c r="J4" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>??ng nh?p ch? nh?p m?t kh?u</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>?ang ? trang ??ng nh?p</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>MatKhauSai123!</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>?? tr?ng t?n ??ng nh?p; nh?p m?t kh?u; nh?n ??ng nh?p</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Kh?ng v?o ???c ?ng d?ng; ti?p t?c ? trang ??ng nh?p</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>submit_password_only</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>

</xml_diff>

<commit_message>
Add TC_LOGIN_005 invalid credentials case
</commit_message>
<xml_diff>
--- a/test_cases/login_test_cases.xlsx
+++ b/test_cases/login_test_cases.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -643,6 +643,58 @@
         </is>
       </c>
       <c r="J5" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>??ng nh?p v?i th?ng tin kh?ng h?p l?</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>?ang ? trang ??ng nh?p</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>automation.invalid@example.com</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>WrongPassword!234</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Nh?p t?i kho?n v? m?t kh?u kh?ng h?p l?; nh?n ??ng nh?p</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Kh?ng v?o ???c ?ng d?ng; ti?p t?c ? trang ??ng nh?p</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>submit_invalid_credentials</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>

</xml_diff>

<commit_message>
Fix Vietnamese text encoding in login test cases
</commit_message>
<xml_diff>
--- a/test_cases/login_test_cases.xlsx
+++ b/test_cases/login_test_cases.xlsx
@@ -483,22 +483,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Ki?m tra trang ??ng nh?p hi?n th? ??y ??</t>
+          <t>Kiểm tra trang đăng nhập hiển thị đầy đủ</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>M? ???c website</t>
+          <t>Mở được website</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>M? URL ??ng nh?p; quan s?t ti?u ??, t?n ??ng nh?p, m?t kh?u v? n?t ??ng nh?p</t>
+          <t>Mở URL đăng nhập; quan sát tiêu đề, tên đăng nhập, mật khẩu và nút đăng nhập</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Hi?n th? ??ng trang ??ng nh?p c?ng c?c tr??ng v? n?t c?n thi?t</t>
+          <t>Hiển thị đúng trang đăng nhập cùng các trường và nút cần thiết</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -525,22 +525,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>??ng nh?p khi b? tr?ng c? t?n ??ng nh?p v? m?t kh?u</t>
+          <t>Đăng nhập khi bỏ trống cả tên đăng nhập và mật khẩu</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>?ang ? trang ??ng nh?p</t>
+          <t>Đang ở trang đăng nhập</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>?? tr?ng hai tr??ng; nh?n ??ng nh?p</t>
+          <t>Để trống hai trường; nhấn Đăng nhập</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Kh?ng v?o ???c ?ng d?ng; ti?p t?c ? trang ??ng nh?p</t>
+          <t>Không vào được ứng dụng; tiếp tục ở trang đăng nhập</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -567,12 +567,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>??ng nh?p ch? nh?p t?n ??ng nh?p</t>
+          <t>Đăng nhập chỉ nhập tên đăng nhập</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>?ang ? trang ??ng nh?p</t>
+          <t>Đang ở trang đăng nhập</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -582,12 +582,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Nh?p t?n ??ng nh?p; ?? tr?ng m?t kh?u; nh?n ??ng nh?p</t>
+          <t>Nhập tên đăng nhập; để trống mật khẩu; nhấn Đăng nhập</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Kh?ng v?o ???c ?ng d?ng; ti?p t?c ? trang ??ng nh?p</t>
+          <t>Không vào được ứng dụng; tiếp tục ở trang đăng nhập</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -614,12 +614,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>??ng nh?p ch? nh?p m?t kh?u</t>
+          <t>Đăng nhập chỉ nhập mật khẩu</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>?ang ? trang ??ng nh?p</t>
+          <t>Đang ở trang đăng nhập</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -629,12 +629,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>?? tr?ng t?n ??ng nh?p; nh?p m?t kh?u; nh?n ??ng nh?p</t>
+          <t>Để trống tên đăng nhập; nhập mật khẩu; nhấn Đăng nhập</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Kh?ng v?o ???c ?ng d?ng; ti?p t?c ? trang ??ng nh?p</t>
+          <t>Không vào được ứng dụng; tiếp tục ở trang đăng nhập</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -661,12 +661,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>??ng nh?p v?i th?ng tin kh?ng h?p l?</t>
+          <t>Đăng nhập với thông tin không hợp lệ</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>?ang ? trang ??ng nh?p</t>
+          <t>Đang ở trang đăng nhập</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -681,12 +681,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Nh?p t?i kho?n v? m?t kh?u kh?ng h?p l?; nh?n ??ng nh?p</t>
+          <t>Nhập tài khoản và mật khẩu không hợp lệ; nhấn Đăng nhập</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Kh?ng v?o ???c ?ng d?ng; ti?p t?c ? trang ??ng nh?p</t>
+          <t>Không vào được ứng dụng; tiếp tục ở trang đăng nhập</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">

</xml_diff>

<commit_message>
Add TC_LOGIN_007 remember me checkbox case
</commit_message>
<xml_diff>
--- a/test_cases/login_test_cases.xlsx
+++ b/test_cases/login_test_cases.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Login" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Login'!$A$1:$J$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Login'!$A$1:$J$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -754,8 +754,50 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Kiểm tra checkbox Ghi nhớ tôi luôn đăng nhập</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Mở trang đăng nhập</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Kiểm tra trạng thái ban đầu; bấm checkbox hai lần</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Checkbox chuyển từ bỏ chọn sang chọn và trở lại</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>remember_me_toggle</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J7"/>
+  <autoFilter ref="A1:J8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add TC_LOGIN_006 password masking case
</commit_message>
<xml_diff>
--- a/test_cases/login_test_cases.xlsx
+++ b/test_cases/login_test_cases.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Login" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Login'!$A$1:$J$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Login'!$A$1:$J$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -415,8 +415,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="27" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="65" customWidth="1" min="7" max="7"/>
+    <col width="65" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -700,8 +712,50 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Kiểm tra mật khẩu được che</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Mở trang đăng nhập</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Quan sát trường mật khẩu</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Trường mật khẩu có type=password</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>password_masked</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J1"/>
+  <autoFilter ref="A1:J7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add TC_LOGIN_009 UTC email sign-in link case
</commit_message>
<xml_diff>
--- a/test_cases/login_test_cases.xlsx
+++ b/test_cases/login_test_cases.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Login" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Login'!$A$1:$J$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Login'!$A$1:$J$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -838,8 +838,50 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Kiểm tra liên kết đăng nhập email UTC</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Mở trang đăng nhập</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Kiểm tra liên kết đăng nhập email UTC</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Liên kết trỏ đến trang xác thực Google UTC</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>google_login_link</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J9"/>
+  <autoFilter ref="A1:J10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add TC_LOGIN_008 password recovery page case
</commit_message>
<xml_diff>
--- a/test_cases/login_test_cases.xlsx
+++ b/test_cases/login_test_cases.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Login" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Login'!$A$1:$J$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Login'!$A$1:$J$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -796,8 +796,50 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Mở trang Lấy lại mật khẩu</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Mở trang đăng nhập</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Bấm liên kết quên mật khẩu</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Mở trang khôi phục có trường email và mã bảo mật</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>forgot_password_link</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J8"/>
+  <autoFilter ref="A1:J9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>